<commit_message>
solve padding and alignment issue , add leave_taken_in_month field in salary sleep data
</commit_message>
<xml_diff>
--- a/salaryData/test14.xlsx
+++ b/salaryData/test14.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>jimit</t>
   </si>
@@ -132,6 +132,9 @@
   </si>
   <si>
     <t>TDS_IT</t>
+  </si>
+  <si>
+    <t>Leave_Taken_In_Month</t>
   </si>
 </sst>
 </file>
@@ -501,7 +504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AC2"/>
+  <dimension ref="A1:AD2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="18" customWidth="1"/>
@@ -510,22 +513,22 @@
     <col min="6" max="6" width="20.7109375" customWidth="1"/>
     <col min="7" max="7" width="20.85546875" customWidth="1"/>
     <col min="8" max="8" width="18.7109375" customWidth="1"/>
-    <col min="9" max="9" width="26.7109375" customWidth="1"/>
-    <col min="10" max="10" width="20.5703125" customWidth="1"/>
-    <col min="11" max="11" width="13.42578125" customWidth="1"/>
-    <col min="12" max="12" width="31.5703125" customWidth="1"/>
-    <col min="13" max="13" width="20.5703125" customWidth="1"/>
-    <col min="15" max="20" width="20.5703125" customWidth="1"/>
-    <col min="22" max="22" width="17.5703125" customWidth="1"/>
-    <col min="23" max="23" width="19" customWidth="1"/>
-    <col min="25" max="25" width="16.28515625" customWidth="1"/>
-    <col min="26" max="26" width="15.42578125" customWidth="1"/>
-    <col min="27" max="27" width="16.42578125" customWidth="1"/>
-    <col min="28" max="28" width="19" customWidth="1"/>
-    <col min="29" max="29" width="16.28515625" customWidth="1"/>
+    <col min="9" max="10" width="26.7109375" customWidth="1"/>
+    <col min="11" max="11" width="20.5703125" customWidth="1"/>
+    <col min="12" max="12" width="13.42578125" customWidth="1"/>
+    <col min="13" max="13" width="31.5703125" customWidth="1"/>
+    <col min="14" max="14" width="20.5703125" customWidth="1"/>
+    <col min="16" max="21" width="20.5703125" customWidth="1"/>
+    <col min="23" max="23" width="17.5703125" customWidth="1"/>
+    <col min="24" max="24" width="19" customWidth="1"/>
+    <col min="26" max="26" width="16.28515625" customWidth="1"/>
+    <col min="27" max="27" width="15.42578125" customWidth="1"/>
+    <col min="28" max="28" width="16.42578125" customWidth="1"/>
+    <col min="29" max="29" width="19" customWidth="1"/>
+    <col min="30" max="30" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:30" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -554,67 +557,70 @@
         <v>12</v>
       </c>
       <c r="J1" t="s">
+        <v>36</v>
+      </c>
+      <c r="K1" t="s">
         <v>13</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>3</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>14</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>22</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>5</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>17</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>33</v>
       </c>
-      <c r="R1" s="4" t="s">
+      <c r="S1" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="S1" s="5" t="s">
+      <c r="T1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="T1" s="5" t="s">
+      <c r="U1" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="4" t="s">
+      <c r="W1" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="6" t="s">
+      <c r="X1" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="X1" s="6" t="s">
+      <c r="Y1" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="Y1" s="7" t="s">
+      <c r="Z1" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="Z1" s="6" t="s">
+      <c r="AA1" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="AA1" s="6" t="s">
+      <c r="AB1" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" t="s">
         <v>28</v>
       </c>
-      <c r="AC1" s="6" t="s">
+      <c r="AD1" s="6" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:30" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2</v>
       </c>
@@ -643,63 +649,66 @@
         <v>1</v>
       </c>
       <c r="J2">
+        <v>2</v>
+      </c>
+      <c r="K2">
         <v>5</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>4</v>
       </c>
-      <c r="L2" s="3">
+      <c r="M2" s="3">
         <v>44743</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>6000</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>2400</v>
       </c>
-      <c r="O2">
+      <c r="P2">
         <v>1600</v>
-      </c>
-      <c r="P2">
-        <v>5000</v>
       </c>
       <c r="Q2">
         <v>5000</v>
       </c>
       <c r="R2">
-        <v>0</v>
+        <v>5000</v>
       </c>
       <c r="S2">
         <v>0</v>
       </c>
       <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
         <v>20000</v>
       </c>
-      <c r="U2">
+      <c r="V2">
         <v>300</v>
       </c>
-      <c r="V2">
+      <c r="W2">
         <v>1200</v>
-      </c>
-      <c r="W2">
-        <v>100</v>
       </c>
       <c r="X2">
         <v>100</v>
       </c>
       <c r="Y2">
+        <v>100</v>
+      </c>
+      <c r="Z2">
         <v>1700</v>
       </c>
-      <c r="Z2">
+      <c r="AA2">
         <v>18300</v>
       </c>
-      <c r="AA2" t="s">
+      <c r="AB2" t="s">
         <v>31</v>
       </c>
-      <c r="AB2" t="s">
+      <c r="AC2" t="s">
         <v>32</v>
       </c>
-      <c r="AC2" s="2">
+      <c r="AD2" s="2">
         <v>44627</v>
       </c>
     </row>

</xml_diff>